<commit_message>
run htss key gen
</commit_message>
<xml_diff>
--- a/tests/birkhoff-test.xlsx
+++ b/tests/birkhoff-test.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\thesis\libs\rust-lib\cggmp21\tests\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7AB58A3E-A5BB-4E97-9BFE-FE2D53136D16}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{860285DC-4D67-4A8D-8DED-16610F8DD0BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{073955CC-5D81-4FB7-B20C-E692441A3FCE}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{073955CC-5D81-4FB7-B20C-E692441A3FCE}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="birkhoff matrix" sheetId="1" r:id="rId1"/>
+    <sheet name="birkhoff coeficient" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="36">
   <si>
     <t>mod_inverse</t>
   </si>
@@ -128,10 +129,22 @@
     <t>2 happy case: identity, normal; 1 unhappy case: singular matrix</t>
   </si>
   <si>
-    <t>DONE (error at multi)inverse_diagonal)</t>
-  </si>
-  <si>
     <t>Diagonal^{-1} * A</t>
+  </si>
+  <si>
+    <t>DONE (error at multi_inverse_diagonal)</t>
+  </si>
+  <si>
+    <t>birkhoff_coefficient</t>
+  </si>
+  <si>
+    <t>get_linear_equation_coefficient_matrix</t>
+  </si>
+  <si>
+    <t>get_coefficient</t>
+  </si>
+  <si>
+    <t>only happy case</t>
   </si>
 </sst>
 </file>
@@ -147,16 +160,15 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <b/>
       <sz val="11"/>
-      <color rgb="FFFF0000"/>
+      <color theme="1"/>
       <name val="Arial"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
       <sz val="11"/>
-      <color theme="1"/>
       <name val="Arial"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -197,12 +209,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
@@ -222,11 +234,14 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -660,11 +675,11 @@
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A5" s="8"/>
-      <c r="B5" s="8"/>
-      <c r="C5" s="8"/>
-      <c r="D5" s="8"/>
-      <c r="E5" s="8"/>
+      <c r="A5" s="7"/>
+      <c r="B5" s="7"/>
+      <c r="C5" s="7"/>
+      <c r="D5" s="7"/>
+      <c r="E5" s="7"/>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="3">
@@ -701,11 +716,11 @@
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A8" s="8"/>
-      <c r="B8" s="8"/>
-      <c r="C8" s="8"/>
-      <c r="D8" s="8"/>
-      <c r="E8" s="8"/>
+      <c r="A8" s="7"/>
+      <c r="B8" s="7"/>
+      <c r="C8" s="7"/>
+      <c r="D8" s="7"/>
+      <c r="E8" s="7"/>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" s="3">
@@ -723,11 +738,11 @@
       <c r="E9" s="4"/>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A10" s="8"/>
-      <c r="B10" s="8"/>
-      <c r="C10" s="8"/>
-      <c r="D10" s="8"/>
-      <c r="E10" s="8"/>
+      <c r="A10" s="7"/>
+      <c r="B10" s="7"/>
+      <c r="C10" s="7"/>
+      <c r="D10" s="7"/>
+      <c r="E10" s="7"/>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" s="3">
@@ -790,11 +805,11 @@
       <c r="E14" s="4"/>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A15" s="8"/>
-      <c r="B15" s="8"/>
-      <c r="C15" s="8"/>
-      <c r="D15" s="8"/>
-      <c r="E15" s="8"/>
+      <c r="A15" s="7"/>
+      <c r="B15" s="7"/>
+      <c r="C15" s="7"/>
+      <c r="D15" s="7"/>
+      <c r="E15" s="7"/>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" s="3">
@@ -827,11 +842,11 @@
       <c r="E17" s="4"/>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A18" s="8"/>
-      <c r="B18" s="8"/>
-      <c r="C18" s="8"/>
-      <c r="D18" s="8"/>
-      <c r="E18" s="8"/>
+      <c r="A18" s="7"/>
+      <c r="B18" s="7"/>
+      <c r="C18" s="7"/>
+      <c r="D18" s="7"/>
+      <c r="E18" s="7"/>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" s="3">
@@ -881,11 +896,11 @@
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A22" s="8"/>
-      <c r="B22" s="8"/>
-      <c r="C22" s="8"/>
-      <c r="D22" s="8"/>
-      <c r="E22" s="8"/>
+      <c r="A22" s="7"/>
+      <c r="B22" s="7"/>
+      <c r="C22" s="7"/>
+      <c r="D22" s="7"/>
+      <c r="E22" s="7"/>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23" s="3">
@@ -936,15 +951,15 @@
         <v>26</v>
       </c>
       <c r="F25" s="1" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A26" s="8"/>
-      <c r="B26" s="8"/>
-      <c r="C26" s="8"/>
-      <c r="D26" s="8"/>
-      <c r="E26" s="8"/>
+      <c r="A26" s="7"/>
+      <c r="B26" s="7"/>
+      <c r="C26" s="7"/>
+      <c r="D26" s="7"/>
+      <c r="E26" s="7"/>
     </row>
     <row r="27" spans="1:6" ht="27.6" x14ac:dyDescent="0.25">
       <c r="A27" s="3">
@@ -964,11 +979,11 @@
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A28" s="8"/>
-      <c r="B28" s="8"/>
-      <c r="C28" s="8"/>
-      <c r="D28" s="8"/>
-      <c r="E28" s="8"/>
+      <c r="A28" s="7"/>
+      <c r="B28" s="7"/>
+      <c r="C28" s="7"/>
+      <c r="D28" s="7"/>
+      <c r="E28" s="7"/>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A29" s="3">
@@ -983,8 +998,8 @@
       <c r="D29" s="5" t="b">
         <v>1</v>
       </c>
-      <c r="E29" s="7" t="s">
-        <v>30</v>
+      <c r="E29" s="8" t="s">
+        <v>31</v>
       </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.25">
@@ -1014,5 +1029,91 @@
     <mergeCell ref="A22:E22"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6D211FD2-DD86-4F41-A191-E3E26089B167}">
+  <dimension ref="A1:E4"/>
+  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="7.8984375" style="9" customWidth="1"/>
+    <col min="2" max="2" width="33.796875" style="9" customWidth="1"/>
+    <col min="3" max="3" width="14.796875" style="9" customWidth="1"/>
+    <col min="4" max="4" width="16.69921875" style="9" customWidth="1"/>
+    <col min="5" max="5" width="26.296875" style="9" customWidth="1"/>
+    <col min="6" max="16384" width="8.796875" style="9"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2" s="3">
+        <v>1</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="C2" s="5" t="b">
+        <v>0</v>
+      </c>
+      <c r="D2" s="5" t="b">
+        <v>0</v>
+      </c>
+      <c r="E2" s="4"/>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3" s="3">
+        <v>2</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="C3" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="D3" s="5" t="b">
+        <v>0</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4" s="3">
+        <v>3</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="C4" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="D4" s="5" t="b">
+        <v>0</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>35</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
log sign with n signers
</commit_message>
<xml_diff>
--- a/tests/birkhoff-test.xlsx
+++ b/tests/birkhoff-test.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\thesis\libs\rust-lib\cggmp21\tests\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{860285DC-4D67-4A8D-8DED-16610F8DD0BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5303394A-3739-4D0D-97D7-2E25A946A3D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{073955CC-5D81-4FB7-B20C-E692441A3FCE}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="37">
   <si>
     <t>mod_inverse</t>
   </si>
@@ -145,6 +145,9 @@
   </si>
   <si>
     <t>only happy case</t>
+  </si>
+  <si>
+    <t>test in various case of rank, threshold and xs</t>
   </si>
 </sst>
 </file>
@@ -1035,7 +1038,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6D211FD2-DD86-4F41-A191-E3E26089B167}">
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="7.8984375" style="9" customWidth="1"/>
@@ -1112,6 +1115,11 @@
         <v>35</v>
       </c>
     </row>
+    <row r="7" spans="1:5" ht="27.6" x14ac:dyDescent="0.25">
+      <c r="B7" s="9" t="s">
+        <v>36</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>